<commit_message>
Sync Oktoberfest dashboard for 2026-10-04
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Desktop\Новая папка\Заполнено_в работу\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676D059A-E334-4F4E-B3BD-71A6E777574B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28488D8F-FCBC-4F0B-B0C8-6CFA112F52CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Октоберфест" sheetId="1" r:id="rId1"/>
@@ -356,7 +356,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -404,6 +404,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -720,6 +721,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B06DD981-710B-49F4-BD8B-F9607C12061A}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B2:G42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1102,7 +1106,7 @@
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="33" t="s">
         <v>27</v>
       </c>
       <c r="C37" s="9"/>
@@ -1165,5 +1169,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="52" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Oktoberfest budget workbook
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28488D8F-FCBC-4F0B-B0C8-6CFA112F52CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0936C4E-125E-442E-905C-8C42C582B48C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -356,7 +356,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -405,6 +405,9 @@
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -732,6 +735,7 @@
     <col min="4" max="4" width="16.7265625" customWidth="1"/>
     <col min="5" max="5" width="12.26953125" customWidth="1"/>
     <col min="6" max="6" width="18.54296875" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
@@ -1133,7 +1137,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="31" t="s">
         <v>30</v>
       </c>
@@ -1148,7 +1152,7 @@
         <f>D39</f>
         <v>220000</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" s="34" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1169,6 +1173,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="52" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Oktoberfest budget and program
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0936C4E-125E-442E-905C-8C42C582B48C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4DDD1D-234F-47E2-82AB-6061D645718C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>Средний чек</t>
   </si>
@@ -119,12 +119,6 @@
     <t>Мастер классы (расходники на 2 дня)</t>
   </si>
   <si>
-    <t>Аренда оборудования (для ведущего и диджея)</t>
-  </si>
-  <si>
-    <t>день</t>
-  </si>
-  <si>
     <t>Оборудование ФУД</t>
   </si>
   <si>
@@ -138,6 +132,21 @@
   </si>
   <si>
     <t>Покупаем один раз и используем на всех фестивалях</t>
+  </si>
+  <si>
+    <t>Аренда оборудования (для ведущего и диджея) за три дня</t>
+  </si>
+  <si>
+    <t>за 3 дня</t>
+  </si>
+  <si>
+    <t>Аренда костюмов ведущему и аниматору</t>
+  </si>
+  <si>
+    <t>Покупка/аренда декора в зону сцены (сено, бочки)</t>
+  </si>
+  <si>
+    <t>Изготовление купонов</t>
   </si>
 </sst>
 </file>
@@ -147,7 +156,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₽&quot;_-;\-* #,##0.00\ &quot;₽&quot;_-;_-* &quot;-&quot;??\ &quot;₽&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +223,15 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -356,7 +374,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -408,6 +426,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -727,7 +752,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:G42"/>
+  <dimension ref="B2:I45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -736,6 +761,7 @@
     <col min="5" max="5" width="12.26953125" customWidth="1"/>
     <col min="6" max="6" width="18.54296875" customWidth="1"/>
     <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="9" max="9" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
@@ -766,7 +792,7 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C5" s="20">
         <v>0.46</v>
@@ -812,7 +838,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="3">
         <f>F17-F22</f>
-        <v>6718671.9148936169</v>
+        <v>7113671.9148936169</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -881,7 +907,7 @@
       <c r="E21" s="12"/>
       <c r="F21" s="25">
         <f>F22</f>
-        <v>5781328.0851063831</v>
+        <v>5386328.0851063831</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.35">
@@ -892,8 +918,8 @@
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="14">
-        <f>F23+F24+F25+F26+F38+F40+F31+F36+F37</f>
-        <v>5781328.0851063831</v>
+        <f>F23+F24+F26+F27+F41+F43+F32+F37+F38</f>
+        <v>5386328.0851063831</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.35">
@@ -919,257 +945,293 @@
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B25" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="29">
-        <f>C2*C3*C4</f>
-        <v>2875000</v>
-      </c>
+      <c r="B25" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="28"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="9" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="29">
-        <f>SUM(F27:F30)</f>
-        <v>1081860</v>
+        <f>C2*C3*C4</f>
+        <v>2875000</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="15">
         <v>12</v>
       </c>
-      <c r="D27" s="16">
-        <v>6500</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F27" s="30">
-        <f>(D27*C27)*1.46*C6</f>
-        <v>341640</v>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="29">
+        <f>SUM(F28:F31)</f>
+        <v>1081860</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" s="15">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D28" s="16">
-        <v>4000</v>
+        <v>6500</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F28" s="30">
         <f>(D28*C28)*1.46*C6</f>
-        <v>105120</v>
+        <v>341640</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C29" s="15">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="D29" s="16">
         <v>4000</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F29" s="30">
         <f>(D29*C29)*1.46*C6</f>
-        <v>438000</v>
+        <v>105120</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C30" s="15">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D30" s="16">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F30" s="30">
         <f>(D30*C30)*1.46*C6</f>
-        <v>197100</v>
+        <v>438000</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B31" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="29">
-        <f>SUM(F32:F35)</f>
-        <v>224468.08510638302</v>
+        <v>16</v>
+      </c>
+      <c r="C31" s="15">
+        <v>10</v>
+      </c>
+      <c r="D31" s="16">
+        <v>4500</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F31" s="30">
+        <f>(D31*C31)*1.46*C6</f>
+        <v>197100</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="15"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="29">
+        <f>SUM(F33:F36)</f>
+        <v>224468.08510638302</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B33" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="15">
+      <c r="C33" s="15">
         <v>1</v>
       </c>
-      <c r="D32" s="16">
+      <c r="D33" s="16">
         <v>4000</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" s="30">
-        <f>(D32*C32*13)/0.94</f>
-        <v>55319.148936170219</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B33" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C33" s="17">
-        <v>4</v>
-      </c>
-      <c r="D33" s="16">
-        <v>2000</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>18</v>
       </c>
       <c r="F33" s="30">
-        <f>(D33*C33*5*C6)/0.94</f>
-        <v>127659.57446808512</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
+        <f>(D33*C33*13)/0.94</f>
+        <v>55319.148936170219</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B34" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C34" s="17">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D34" s="16">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="E34" s="9" t="s">
         <v>18</v>
       </c>
       <c r="F34" s="30">
-        <f>((D34*C34)*3)/0.94</f>
-        <v>15957.44680851064</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
+        <f>(D34*C34*5*C6)/0.94</f>
+        <v>127659.57446808512</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B35" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C35" s="17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="16">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>18</v>
       </c>
       <c r="F35" s="30">
-        <f>((C35*D35)*6)/0.94</f>
+        <f>((D35*C35)*3)/0.94</f>
+        <v>15957.44680851064</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B36" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" s="17">
+        <v>2</v>
+      </c>
+      <c r="D36" s="16">
+        <v>2000</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="30">
+        <f>((C36*D36)*6)/0.94</f>
         <v>25531.914893617024</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B36" s="9" t="s">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B37" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="29">
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="29">
         <v>50000</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B37" s="33" t="s">
+    <row r="38" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B38" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="9"/>
+      <c r="D38" s="16">
+        <f>280000+165000</f>
+        <v>445000</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" s="29">
+        <f>D38</f>
+        <v>445000</v>
+      </c>
+      <c r="I38" s="35"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B39" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="17">
+        <v>5</v>
+      </c>
+      <c r="D39" s="37"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="38">
+        <f>D39*C39*C6</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="35"/>
+    </row>
+    <row r="40" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B40" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="17"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="38"/>
+      <c r="I40" s="35"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B41" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="16">
-        <v>280000</v>
-      </c>
-      <c r="E37" s="9" t="s">
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="29">
+        <f>F42</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="F37" s="29">
-        <f>D37*C6</f>
-        <v>840000</v>
-      </c>
-    </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B38" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="29">
-        <f>F39</f>
+      <c r="C42" s="15">
+        <v>3</v>
+      </c>
+      <c r="D42" s="10">
         <v>220000</v>
       </c>
-    </row>
-    <row r="39" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="C39" s="15">
-        <v>3</v>
-      </c>
-      <c r="D39" s="10">
+      <c r="E42" s="9"/>
+      <c r="F42" s="29">
+        <f>D42</f>
         <v>220000</v>
       </c>
-      <c r="E39" s="9"/>
-      <c r="F39" s="29">
-        <f>D39</f>
-        <v>220000</v>
-      </c>
-      <c r="G39" s="34" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B40" s="9" t="s">
+      <c r="G42" s="34" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B43" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="29">
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="29">
         <f>C8*C6</f>
         <v>60000</v>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="F42" s="18"/>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="F45" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Sync updated Oktoberfest budget
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D4DDD1D-234F-47E2-82AB-6061D645718C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C56C97-1361-4A1C-BC11-1B93586FB9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Средний чек</t>
   </si>
@@ -140,13 +140,19 @@
     <t>за 3 дня</t>
   </si>
   <si>
-    <t>Аренда костюмов ведущему и аниматору</t>
-  </si>
-  <si>
-    <t>Покупка/аренда декора в зону сцены (сено, бочки)</t>
-  </si>
-  <si>
-    <t>Изготовление купонов</t>
+    <t>посчитать маржу3 и маржинальность</t>
+  </si>
+  <si>
+    <t>Покупка/аренда декора в зону сцены ( бочки-столы/бочки, гирлянда)</t>
+  </si>
+  <si>
+    <t>Покупка костюмов аниматорам+ведущий</t>
+  </si>
+  <si>
+    <t>сено берем у альпак</t>
+  </si>
+  <si>
+    <t>Изготовление билетов и купонов (с доставкой)</t>
   </si>
 </sst>
 </file>
@@ -374,7 +380,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -433,6 +439,7 @@
     <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -752,7 +759,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I45"/>
+  <dimension ref="B2:M45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -838,7 +845,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="3">
         <f>F17-F22</f>
-        <v>7113671.9148936169</v>
+        <v>7371671.9148936169</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -860,7 +867,7 @@
         <v>12500000</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B17" s="7" t="s">
         <v>7</v>
       </c>
@@ -872,7 +879,7 @@
         <v>12500000</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B18" s="9" t="s">
         <v>8</v>
       </c>
@@ -884,21 +891,21 @@
         <v>12500000</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B19" s="24"/>
       <c r="C19" s="24"/>
       <c r="D19" s="24"/>
       <c r="E19" s="24"/>
       <c r="F19" s="9"/>
     </row>
-    <row r="20" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
       <c r="D20" s="24"/>
       <c r="E20" s="24"/>
       <c r="F20" s="24"/>
     </row>
-    <row r="21" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="11" t="s">
         <v>9</v>
       </c>
@@ -907,10 +914,10 @@
       <c r="E21" s="12"/>
       <c r="F21" s="25">
         <f>F22</f>
-        <v>5386328.0851063831</v>
-      </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+        <v>5128328.0851063831</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B22" s="13" t="s">
         <v>10</v>
       </c>
@@ -919,10 +926,10 @@
       <c r="E22" s="13"/>
       <c r="F22" s="14">
         <f>F23+F24+F26+F27+F41+F43+F32+F37+F38</f>
-        <v>5386328.0851063831</v>
-      </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+        <v>5128328.0851063831</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B23" s="26" t="s">
         <v>11</v>
       </c>
@@ -933,7 +940,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B24" s="26" t="s">
         <v>20</v>
       </c>
@@ -944,16 +951,22 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B25" s="39" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
+      <c r="D25" s="37">
+        <f>6200+500+2500</f>
+        <v>9200</v>
+      </c>
       <c r="E25" s="27"/>
-      <c r="F25" s="28"/>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F25" s="40">
+        <f>D25</f>
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B26" s="9" t="s">
         <v>8</v>
       </c>
@@ -965,7 +978,7 @@
         <v>2875000</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B27" s="9" t="s">
         <v>12</v>
       </c>
@@ -977,7 +990,7 @@
         <v>1081860</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B28" s="9" t="s">
         <v>13</v>
       </c>
@@ -995,7 +1008,7 @@
         <v>341640</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B29" s="9" t="s">
         <v>14</v>
       </c>
@@ -1013,7 +1026,7 @@
         <v>105120</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B30" s="9" t="s">
         <v>15</v>
       </c>
@@ -1030,8 +1043,11 @@
         <f>(D30*C30)*1.46*C6</f>
         <v>438000</v>
       </c>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="M30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B31" s="9" t="s">
         <v>16</v>
       </c>
@@ -1049,7 +1065,7 @@
         <v>197100</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B32" s="9" t="s">
         <v>17</v>
       </c>
@@ -1138,7 +1154,7 @@
         <v>26</v>
       </c>
       <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
+      <c r="D37" s="37"/>
       <c r="E37" s="9"/>
       <c r="F37" s="29">
         <v>50000</v>
@@ -1150,30 +1166,34 @@
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="16">
-        <f>280000+165000</f>
-        <v>445000</v>
+        <f>187000</f>
+        <v>187000</v>
       </c>
       <c r="E38" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F38" s="29">
+      <c r="F38" s="38">
         <f>D38</f>
-        <v>445000</v>
+        <v>187000</v>
       </c>
       <c r="I38" s="35"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B39" s="36" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C39" s="17">
         <v>5</v>
       </c>
-      <c r="D39" s="37"/>
-      <c r="E39" s="33"/>
+      <c r="D39" s="37">
+        <v>15000</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="F39" s="38">
-        <f>D39*C39*C6</f>
-        <v>0</v>
+        <f>D39</f>
+        <v>15000</v>
       </c>
       <c r="I39" s="35"/>
     </row>
@@ -1182,9 +1202,20 @@
         <v>35</v>
       </c>
       <c r="C40" s="17"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="33"/>
-      <c r="F40" s="38"/>
+      <c r="D40" s="37">
+        <f>54000+5000</f>
+        <v>59000</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" s="38">
+        <f>D40</f>
+        <v>59000</v>
+      </c>
+      <c r="G40" t="s">
+        <v>37</v>
+      </c>
       <c r="I40" s="35"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Refresh Oktoberfest sources and add detailed timing and program
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06C56C97-1361-4A1C-BC11-1B93586FB9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0BD782-FA14-452F-BA50-98F7398AF127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -110,9 +110,6 @@
     <t>Аниматоры (по 5 часов)</t>
   </si>
   <si>
-    <t>Диджей (3 часа)</t>
-  </si>
-  <si>
     <t>Мастер классы (аниматоры 6 часов)</t>
   </si>
   <si>
@@ -153,6 +150,33 @@
   </si>
   <si>
     <t>Изготовление билетов и купонов (с доставкой)</t>
+  </si>
+  <si>
+    <r>
+      <t>Диджей (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> часа)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -380,7 +404,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -440,6 +464,10 @@
     <xf numFmtId="44" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -799,7 +827,7 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" s="20">
         <v>0.46</v>
@@ -845,7 +873,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="3">
         <f>F17-F22</f>
-        <v>7371671.9148936169</v>
+        <v>7376991.0638297871</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -914,7 +942,7 @@
       <c r="E21" s="12"/>
       <c r="F21" s="25">
         <f>F22</f>
-        <v>5128328.0851063831</v>
+        <v>5123008.9361702129</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.35">
@@ -926,7 +954,7 @@
       <c r="E22" s="13"/>
       <c r="F22" s="14">
         <f>F23+F24+F26+F27+F41+F43+F32+F37+F38</f>
-        <v>5128328.0851063831</v>
+        <v>5123008.9361702129</v>
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.35">
@@ -953,7 +981,7 @@
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B25" s="39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" s="27"/>
       <c r="D25" s="37">
@@ -1001,7 +1029,7 @@
         <v>6500</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F28" s="30">
         <f>(D28*C28)*1.46*C6</f>
@@ -1019,7 +1047,7 @@
         <v>4000</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F29" s="30">
         <f>(D29*C29)*1.46*C6</f>
@@ -1037,14 +1065,14 @@
         <v>4000</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F30" s="30">
         <f>(D30*C30)*1.46*C6</f>
         <v>438000</v>
       </c>
       <c r="M30" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.35">
@@ -1058,7 +1086,7 @@
         <v>4500</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F31" s="30">
         <f>(D31*C31)*1.46*C6</f>
@@ -1074,7 +1102,7 @@
       <c r="E32" s="16"/>
       <c r="F32" s="29">
         <f>SUM(F33:F36)</f>
-        <v>224468.08510638302</v>
+        <v>219148.93617021281</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.35">
@@ -1115,7 +1143,7 @@
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B35" s="9" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C35" s="17">
         <v>1</v>
@@ -1126,14 +1154,14 @@
       <c r="E35" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F35" s="30">
-        <f>((D35*C35)*3)/0.94</f>
-        <v>15957.44680851064</v>
+      <c r="F35" s="42">
+        <f>((D35*C35)*2)/0.94</f>
+        <v>10638.297872340427</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C36" s="17">
         <v>2</v>
@@ -1151,7 +1179,7 @@
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B37" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="37"/>
@@ -1161,8 +1189,8 @@
       </c>
     </row>
     <row r="38" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B38" s="36" t="s">
-        <v>32</v>
+      <c r="B38" s="41" t="s">
+        <v>31</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="16">
@@ -1170,7 +1198,7 @@
         <v>187000</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F38" s="38">
         <f>D38</f>
@@ -1180,7 +1208,7 @@
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B39" s="36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C39" s="17">
         <v>5</v>
@@ -1189,7 +1217,7 @@
         <v>15000</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F39" s="38">
         <f>D39</f>
@@ -1199,7 +1227,7 @@
     </row>
     <row r="40" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B40" s="36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="37">
@@ -1207,20 +1235,20 @@
         <v>59000</v>
       </c>
       <c r="E40" s="33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F40" s="38">
         <f>D40</f>
         <v>59000</v>
       </c>
       <c r="G40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I40" s="35"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B41" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
@@ -1232,7 +1260,7 @@
     </row>
     <row r="42" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C42" s="15">
         <v>3</v>
@@ -1246,7 +1274,7 @@
         <v>220000</v>
       </c>
       <c r="G42" s="34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Refresh schedule budget and timing from latest source files
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0BD782-FA14-452F-BA50-98F7398AF127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8F0987-AAD5-4841-A6D7-6DD3BF5F6986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Октоберфест" sheetId="1" r:id="rId1"/>
@@ -795,7 +795,7 @@
     <col min="4" max="4" width="16.7265625" customWidth="1"/>
     <col min="5" max="5" width="12.26953125" customWidth="1"/>
     <col min="6" max="6" width="18.54296875" customWidth="1"/>
-    <col min="7" max="7" width="48" customWidth="1"/>
+    <col min="7" max="7" width="69.7265625" customWidth="1"/>
     <col min="9" max="9" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Show tickets meals risks and sync budget
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8F0987-AAD5-4841-A6D7-6DD3BF5F6986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A61B373-A5EA-4C50-AFE8-AA6DF5F2F66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Октоберфест" sheetId="1" r:id="rId1"/>
@@ -140,9 +140,6 @@
     <t>посчитать маржу3 и маржинальность</t>
   </si>
   <si>
-    <t>Покупка/аренда декора в зону сцены ( бочки-столы/бочки, гирлянда)</t>
-  </si>
-  <si>
     <t>Покупка костюмов аниматорам+ведущий</t>
   </si>
   <si>
@@ -152,31 +149,10 @@
     <t>Изготовление билетов и купонов (с доставкой)</t>
   </si>
   <si>
-    <r>
-      <t>Диджей (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> часа)</t>
-    </r>
+    <t>Диджей (2 часа)</t>
+  </si>
+  <si>
+    <t>Покупка/аренда декора в зону сцены ( бочки-столы (8шт), гирлянда)</t>
   </si>
 </sst>
 </file>
@@ -186,7 +162,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₽&quot;_-;\-* #,##0.00\ &quot;₽&quot;_-;_-* &quot;-&quot;??\ &quot;₽&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,24 +173,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -255,8 +213,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -404,70 +361,60 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="5" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="3" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -787,7 +734,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M45"/>
+  <dimension ref="B2:M42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -803,7 +750,7 @@
       <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="19">
+      <c r="C2" s="2">
         <v>2500</v>
       </c>
     </row>
@@ -819,21 +766,21 @@
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="3">
         <v>0.23</v>
       </c>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="3">
         <v>0.46</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
@@ -855,442 +802,442 @@
       <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="2">
         <v>20000</v>
       </c>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-    </row>
-    <row r="13" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="F13" s="21"/>
-    </row>
-    <row r="14" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="1" t="s">
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="10" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="3">
-        <f>F17-F22</f>
-        <v>7376991.0638297871</v>
-      </c>
-    </row>
-    <row r="15" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="22"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="14">
+        <f>F14-F19</f>
+        <v>7293791.0638297871</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="16"/>
+    </row>
+    <row r="13" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="19">
+        <f>F14</f>
+        <v>12500000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B14" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="21">
+        <f>SUM(F15:F17)</f>
+        <v>12500000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B15" s="22" t="s">
+        <v>8</v>
+      </c>
       <c r="C15" s="22"/>
       <c r="D15" s="22"/>
       <c r="E15" s="22"/>
-      <c r="F15" s="23"/>
-    </row>
-    <row r="16" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="6">
-        <f>F17</f>
-        <v>12500000</v>
-      </c>
-    </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B17" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="8">
-        <f>SUM(F18:F20)</f>
-        <v>12500000</v>
-      </c>
-    </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B18" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="10">
+      <c r="F15" s="7">
         <f>C2*C3</f>
         <v>12500000</v>
       </c>
     </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="22"/>
+    </row>
+    <row r="17" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+    </row>
+    <row r="18" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="26">
+        <f>F19</f>
+        <v>5206208.9361702129</v>
+      </c>
+    </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="9"/>
-    </row>
-    <row r="20" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-    </row>
-    <row r="21" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="25">
-        <f>F22</f>
-        <v>5123008.9361702129</v>
+      <c r="B19" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="28">
+        <f>F20+F21+F22+F23+F24+F38+F40+F29+F34+F35+F36+F37</f>
+        <v>5206208.9361702129</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B20" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="5">
+        <v>400000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B21" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="5">
+        <v>30000</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B22" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="14">
-        <f>F23+F24+F26+F27+F41+F43+F32+F37+F38</f>
-        <v>5123008.9361702129</v>
-      </c>
-    </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B23" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="28">
-        <v>400000</v>
-      </c>
-    </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B24" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="28">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B25" s="39" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="27"/>
-      <c r="D25" s="37">
+      <c r="B22" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="30"/>
+      <c r="D22" s="31">
         <f>6200+500+2500</f>
         <v>9200</v>
       </c>
-      <c r="E25" s="27"/>
-      <c r="F25" s="40">
-        <f>D25</f>
+      <c r="E22" s="30"/>
+      <c r="F22" s="5">
+        <f>D22</f>
         <v>9200</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B26" s="9" t="s">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B23" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="29">
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="6">
         <f>C2*C3*C4</f>
         <v>2875000</v>
       </c>
     </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B24" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="6">
+        <f>SUM(F25:F28)</f>
+        <v>1081860</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B25" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="32">
+        <v>12</v>
+      </c>
+      <c r="D25" s="31">
+        <v>6500</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25" s="7">
+        <f>(D25*C25)*1.46*C6</f>
+        <v>341640</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B26" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="32">
+        <v>6</v>
+      </c>
+      <c r="D26" s="31">
+        <v>4000</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F26" s="7">
+        <f>(D26*C26)*1.46*C6</f>
+        <v>105120</v>
+      </c>
+    </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B27" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="29">
-        <f>SUM(F28:F31)</f>
-        <v>1081860</v>
+      <c r="B27" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="32">
+        <v>25</v>
+      </c>
+      <c r="D27" s="31">
+        <v>4000</v>
+      </c>
+      <c r="E27" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27" s="7">
+        <f>(D27*C27)*1.46*C6</f>
+        <v>438000</v>
+      </c>
+      <c r="M27" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B28" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="15">
-        <v>12</v>
-      </c>
-      <c r="D28" s="16">
-        <v>6500</v>
-      </c>
-      <c r="E28" s="9" t="s">
+      <c r="B28" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="32">
+        <v>10</v>
+      </c>
+      <c r="D28" s="31">
+        <v>4500</v>
+      </c>
+      <c r="E28" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="30">
+      <c r="F28" s="7">
         <f>(D28*C28)*1.46*C6</f>
-        <v>341640</v>
+        <v>197100</v>
       </c>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B29" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C29" s="15">
-        <v>6</v>
-      </c>
-      <c r="D29" s="16">
+      <c r="B29" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="32"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="6">
+        <f>SUM(F30:F33)</f>
+        <v>219148.93617021281</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B30" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" s="32">
+        <v>1</v>
+      </c>
+      <c r="D30" s="31">
         <v>4000</v>
       </c>
-      <c r="E29" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F29" s="30">
-        <f>(D29*C29)*1.46*C6</f>
-        <v>105120</v>
-      </c>
-    </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B30" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C30" s="15">
+      <c r="E30" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="7">
+        <f>(D30*C30*13)/0.94</f>
+        <v>55319.148936170219</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B31" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="33">
+        <v>4</v>
+      </c>
+      <c r="D31" s="31">
+        <v>2000</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="7">
+        <f>(D31*C31*5*C6)/0.94</f>
+        <v>127659.57446808512</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B32" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="33">
+        <v>1</v>
+      </c>
+      <c r="D32" s="31">
+        <v>5000</v>
+      </c>
+      <c r="E32" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="7">
+        <f>((D32*C32)*2)/0.94</f>
+        <v>10638.297872340427</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B33" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" s="33">
+        <v>2</v>
+      </c>
+      <c r="D33" s="31">
+        <v>2000</v>
+      </c>
+      <c r="E33" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="7">
+        <f>((C33*D33)*6)/0.94</f>
+        <v>25531.914893617024</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B34" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="16">
-        <v>4000</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F30" s="30">
-        <f>(D30*C30)*1.46*C6</f>
-        <v>438000</v>
-      </c>
-      <c r="M30" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B31" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="15">
-        <v>10</v>
-      </c>
-      <c r="D31" s="16">
-        <v>4500</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F31" s="30">
-        <f>(D31*C31)*1.46*C6</f>
-        <v>197100</v>
-      </c>
-    </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B32" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="29">
-        <f>SUM(F33:F36)</f>
-        <v>219148.93617021281</v>
-      </c>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B33" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C33" s="15">
-        <v>1</v>
-      </c>
-      <c r="D33" s="16">
-        <v>4000</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F33" s="30">
-        <f>(D33*C33*13)/0.94</f>
-        <v>55319.148936170219</v>
-      </c>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B34" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C34" s="17">
-        <v>4</v>
-      </c>
-      <c r="D34" s="16">
-        <v>2000</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F34" s="30">
-        <f>(D34*C34*5*C6)/0.94</f>
-        <v>127659.57446808512</v>
-      </c>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B35" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C35" s="17">
-        <v>1</v>
-      </c>
-      <c r="D35" s="16">
-        <v>5000</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F35" s="42">
-        <f>((D35*C35)*2)/0.94</f>
-        <v>10638.297872340427</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B36" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C36" s="17">
-        <v>2</v>
-      </c>
-      <c r="D36" s="16">
-        <v>2000</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F36" s="30">
-        <f>((C36*D36)*6)/0.94</f>
-        <v>25531.914893617024</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B37" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C37" s="9"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="29">
+      <c r="C34" s="22"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="6">
         <v>50000</v>
       </c>
     </row>
-    <row r="38" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B38" s="41" t="s">
+    <row r="35" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B35" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C38" s="9"/>
-      <c r="D38" s="16">
+      <c r="C35" s="22"/>
+      <c r="D35" s="31">
         <f>187000</f>
         <v>187000</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="E35" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="F38" s="38">
-        <f>D38</f>
+      <c r="F35" s="6">
+        <f>D35</f>
         <v>187000</v>
       </c>
-      <c r="I38" s="35"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B39" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="17">
+      <c r="I35" s="10"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B36" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="33">
         <v>5</v>
       </c>
-      <c r="D39" s="37">
+      <c r="D36" s="31">
         <v>15000</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E36" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="F39" s="38">
-        <f>D39</f>
+      <c r="F36" s="6">
+        <f>D36</f>
         <v>15000</v>
       </c>
-      <c r="I39" s="35"/>
-    </row>
-    <row r="40" spans="2:9" ht="29" x14ac:dyDescent="0.35">
-      <c r="B40" s="36" t="s">
-        <v>34</v>
-      </c>
-      <c r="C40" s="17"/>
-      <c r="D40" s="37">
+      <c r="I36" s="10"/>
+    </row>
+    <row r="37" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B37" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="33"/>
+      <c r="D37" s="31">
         <f>54000+5000</f>
         <v>59000</v>
       </c>
-      <c r="E40" s="33" t="s">
+      <c r="E37" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="F40" s="38">
-        <f>D40</f>
+      <c r="F37" s="6">
+        <f>D37</f>
         <v>59000</v>
       </c>
-      <c r="G40" t="s">
-        <v>36</v>
-      </c>
-      <c r="I40" s="35"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B41" s="9" t="s">
+      <c r="G37" t="s">
+        <v>35</v>
+      </c>
+      <c r="I37" s="10"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B38" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C41" s="9"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="29">
-        <f>F42</f>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="6">
+        <f>F39</f>
         <v>220000</v>
       </c>
     </row>
-    <row r="42" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="31" t="s">
+    <row r="39" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="C42" s="15">
+      <c r="C39" s="32">
         <v>3</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D39" s="7">
         <v>220000</v>
       </c>
-      <c r="E42" s="9"/>
-      <c r="F42" s="29">
-        <f>D42</f>
+      <c r="E39" s="22"/>
+      <c r="F39" s="6">
+        <f>D39</f>
         <v>220000</v>
       </c>
-      <c r="G42" s="34" t="s">
+      <c r="G39" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B43" s="9" t="s">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B40" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="C43" s="9"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="29">
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="6">
         <f>C8*C6</f>
         <v>60000</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="F45" s="18"/>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="F42" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Sync updated Oktoberfest sources
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A61B373-A5EA-4C50-AFE8-AA6DF5F2F66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2862B1EC-7BF2-4444-8096-C79B372EBF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>Средний чек</t>
   </si>
@@ -135,9 +135,6 @@
   </si>
   <si>
     <t>за 3 дня</t>
-  </si>
-  <si>
-    <t>посчитать маржу3 и маржинальность</t>
   </si>
   <si>
     <t>Покупка костюмов аниматорам+ведущий</t>
@@ -734,7 +731,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M42"/>
+  <dimension ref="B2:I42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -873,14 +870,14 @@
       <c r="E16" s="23"/>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
       <c r="D17" s="23"/>
       <c r="E17" s="23"/>
       <c r="F17" s="23"/>
     </row>
-    <row r="18" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="24" t="s">
         <v>9</v>
       </c>
@@ -892,7 +889,7 @@
         <v>5206208.9361702129</v>
       </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="27" t="s">
         <v>10</v>
       </c>
@@ -904,7 +901,7 @@
         <v>5206208.9361702129</v>
       </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>11</v>
       </c>
@@ -915,7 +912,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>20</v>
       </c>
@@ -926,9 +923,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="31">
@@ -941,7 +938,7 @@
         <v>9200</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="22" t="s">
         <v>8</v>
       </c>
@@ -953,7 +950,7 @@
         <v>2875000</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="22" t="s">
         <v>12</v>
       </c>
@@ -965,7 +962,7 @@
         <v>1081860</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="22" t="s">
         <v>13</v>
       </c>
@@ -983,7 +980,7 @@
         <v>341640</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="22" t="s">
         <v>14</v>
       </c>
@@ -1001,7 +998,7 @@
         <v>105120</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="22" t="s">
         <v>15</v>
       </c>
@@ -1018,11 +1015,8 @@
         <f>(D27*C27)*1.46*C6</f>
         <v>438000</v>
       </c>
-      <c r="M27" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="22" t="s">
         <v>16</v>
       </c>
@@ -1040,7 +1034,7 @@
         <v>197100</v>
       </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="22" t="s">
         <v>17</v>
       </c>
@@ -1052,7 +1046,7 @@
         <v>219148.93617021281</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="22" t="s">
         <v>22</v>
       </c>
@@ -1070,7 +1064,7 @@
         <v>55319.148936170219</v>
       </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B31" s="22" t="s">
         <v>23</v>
       </c>
@@ -1088,9 +1082,9 @@
         <v>127659.57446808512</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C32" s="33">
         <v>1</v>
@@ -1155,7 +1149,7 @@
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C36" s="33">
         <v>5</v>
@@ -1174,7 +1168,7 @@
     </row>
     <row r="37" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B37" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C37" s="33"/>
       <c r="D37" s="31">
@@ -1189,7 +1183,7 @@
         <v>59000</v>
       </c>
       <c r="G37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I37" s="10"/>
     </row>
@@ -1241,6 +1235,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="32" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "Sync updated Oktoberfest sources"
This reverts commit 38a7db818f19fc92cfe789c8bd496d3d770add70.
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2862B1EC-7BF2-4444-8096-C79B372EBF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A61B373-A5EA-4C50-AFE8-AA6DF5F2F66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Средний чек</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>за 3 дня</t>
+  </si>
+  <si>
+    <t>посчитать маржу3 и маржинальность</t>
   </si>
   <si>
     <t>Покупка костюмов аниматорам+ведущий</t>
@@ -731,7 +734,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I42"/>
+  <dimension ref="B2:M42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -870,14 +873,14 @@
       <c r="E16" s="23"/>
       <c r="F16" s="22"/>
     </row>
-    <row r="17" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
       <c r="D17" s="23"/>
       <c r="E17" s="23"/>
       <c r="F17" s="23"/>
     </row>
-    <row r="18" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="24" t="s">
         <v>9</v>
       </c>
@@ -889,7 +892,7 @@
         <v>5206208.9361702129</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B19" s="27" t="s">
         <v>10</v>
       </c>
@@ -901,7 +904,7 @@
         <v>5206208.9361702129</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>11</v>
       </c>
@@ -912,7 +915,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>20</v>
       </c>
@@ -923,9 +926,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="31">
@@ -938,7 +941,7 @@
         <v>9200</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B23" s="22" t="s">
         <v>8</v>
       </c>
@@ -950,7 +953,7 @@
         <v>2875000</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B24" s="22" t="s">
         <v>12</v>
       </c>
@@ -962,7 +965,7 @@
         <v>1081860</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B25" s="22" t="s">
         <v>13</v>
       </c>
@@ -980,7 +983,7 @@
         <v>341640</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B26" s="22" t="s">
         <v>14</v>
       </c>
@@ -998,7 +1001,7 @@
         <v>105120</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B27" s="22" t="s">
         <v>15</v>
       </c>
@@ -1015,8 +1018,11 @@
         <f>(D27*C27)*1.46*C6</f>
         <v>438000</v>
       </c>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="M27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B28" s="22" t="s">
         <v>16</v>
       </c>
@@ -1034,7 +1040,7 @@
         <v>197100</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B29" s="22" t="s">
         <v>17</v>
       </c>
@@ -1046,7 +1052,7 @@
         <v>219148.93617021281</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B30" s="22" t="s">
         <v>22</v>
       </c>
@@ -1064,7 +1070,7 @@
         <v>55319.148936170219</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B31" s="22" t="s">
         <v>23</v>
       </c>
@@ -1082,9 +1088,9 @@
         <v>127659.57446808512</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B32" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C32" s="33">
         <v>1</v>
@@ -1149,7 +1155,7 @@
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C36" s="33">
         <v>5</v>
@@ -1168,7 +1174,7 @@
     </row>
     <row r="37" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B37" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C37" s="33"/>
       <c r="D37" s="31">
@@ -1183,7 +1189,7 @@
         <v>59000</v>
       </c>
       <c r="G37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I37" s="10"/>
     </row>
@@ -1235,6 +1241,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="32" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reapply "Sync updated Oktoberfest sources"
This reverts commit 25addfc407688619ab24cb9f932efcc6b158b515.
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A61B373-A5EA-4C50-AFE8-AA6DF5F2F66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D343EF1A-77EF-4541-A592-633788F8BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>Средний чек</t>
   </si>
@@ -135,9 +135,6 @@
   </si>
   <si>
     <t>за 3 дня</t>
-  </si>
-  <si>
-    <t>посчитать маржу3 и маржинальность</t>
   </si>
   <si>
     <t>Покупка костюмов аниматорам+ведущий</t>
@@ -252,7 +249,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -353,6 +350,34 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -382,25 +407,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="6" fillId="4" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -415,6 +433,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="44" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Денежный" xfId="1" builtinId="4"/>
@@ -734,7 +759,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M42"/>
+  <dimension ref="B2:I42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -818,164 +843,164 @@
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>
-      <c r="F11" s="14">
+      <c r="F11" s="32">
         <f>F14-F19</f>
-        <v>7293791.0638297871</v>
+        <v>7281911.0638297871</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="16"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="15"/>
     </row>
     <row r="13" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="19">
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="33">
         <f>F14</f>
         <v>12500000</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="21">
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="19">
         <f>SUM(F15:F17)</f>
         <v>12500000</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
       <c r="F15" s="7">
         <f>C2*C3</f>
         <v>12500000</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="22"/>
-    </row>
-    <row r="17" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-    </row>
-    <row r="18" spans="2:13" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="24" t="s">
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="20"/>
+    </row>
+    <row r="17" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+    </row>
+    <row r="18" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="26">
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="34">
         <f>F19</f>
-        <v>5206208.9361702129</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B19" s="27" t="s">
+        <v>5218088.9361702129</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28">
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="25">
         <f>F20+F21+F22+F23+F24+F38+F40+F29+F34+F35+F36+F37</f>
-        <v>5206208.9361702129</v>
-      </c>
-    </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
+        <v>5218088.9361702129</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B20" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
       <c r="F20" s="5">
         <v>400000</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B21" s="29" t="s">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
       <c r="F21" s="5">
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B22" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="31">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="27"/>
+      <c r="D22" s="28">
         <f>6200+500+2500</f>
         <v>9200</v>
       </c>
-      <c r="E22" s="30"/>
+      <c r="E22" s="27"/>
       <c r="F22" s="5">
         <f>D22</f>
         <v>9200</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B23" s="22" t="s">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
       <c r="F23" s="6">
         <f>C2*C3*C4</f>
         <v>2875000</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B24" s="22" t="s">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
       <c r="F24" s="6">
         <f>SUM(F25:F28)</f>
         <v>1081860</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B25" s="22" t="s">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B25" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="32">
+      <c r="C25" s="29">
         <v>12</v>
       </c>
-      <c r="D25" s="31">
+      <c r="D25" s="28">
         <v>6500</v>
       </c>
-      <c r="E25" s="22" t="s">
+      <c r="E25" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F25" s="7">
@@ -983,17 +1008,17 @@
         <v>341640</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B26" s="22" t="s">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B26" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="32">
+      <c r="C26" s="29">
         <v>6</v>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="28">
         <v>4000</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F26" s="7">
@@ -1001,38 +1026,35 @@
         <v>105120</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B27" s="22" t="s">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B27" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="29">
         <v>25</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="28">
         <v>4000</v>
       </c>
-      <c r="E27" s="22" t="s">
+      <c r="E27" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F27" s="7">
         <f>(D27*C27)*1.46*C6</f>
         <v>438000</v>
       </c>
-      <c r="M27" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B28" s="22" t="s">
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B28" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="29">
         <v>10</v>
       </c>
-      <c r="D28" s="31">
+      <c r="D28" s="28">
         <v>4500</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="20" t="s">
         <v>29</v>
       </c>
       <c r="F28" s="7">
@@ -1040,29 +1062,29 @@
         <v>197100</v>
       </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B29" s="22" t="s">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B29" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="32"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
       <c r="F29" s="6">
         <f>SUM(F30:F33)</f>
         <v>219148.93617021281</v>
       </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B30" s="22" t="s">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B30" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="29">
         <v>1</v>
       </c>
-      <c r="D30" s="31">
+      <c r="D30" s="28">
         <v>4000</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F30" s="7">
@@ -1070,17 +1092,17 @@
         <v>55319.148936170219</v>
       </c>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B31" s="22" t="s">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B31" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C31" s="33">
+      <c r="C31" s="30">
         <v>4</v>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="28">
         <v>2000</v>
       </c>
-      <c r="E31" s="22" t="s">
+      <c r="E31" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F31" s="7">
@@ -1088,17 +1110,17 @@
         <v>127659.57446808512</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B32" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" s="33">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B32" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" s="30">
         <v>1</v>
       </c>
-      <c r="D32" s="31">
+      <c r="D32" s="28">
         <v>5000</v>
       </c>
-      <c r="E32" s="22" t="s">
+      <c r="E32" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F32" s="7">
@@ -1107,16 +1129,16 @@
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C33" s="33">
+      <c r="C33" s="30">
         <v>2</v>
       </c>
-      <c r="D33" s="31">
+      <c r="D33" s="28">
         <v>2000</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F33" s="7">
@@ -1125,12 +1147,12 @@
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="22"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="20"/>
       <c r="F34" s="6">
         <v>50000</v>
       </c>
@@ -1139,12 +1161,12 @@
       <c r="B35" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="22"/>
-      <c r="D35" s="31">
+      <c r="C35" s="20"/>
+      <c r="D35" s="28">
         <f>187000</f>
         <v>187000</v>
       </c>
-      <c r="E35" s="22" t="s">
+      <c r="E35" s="20" t="s">
         <v>32</v>
       </c>
       <c r="F35" s="6">
@@ -1155,15 +1177,15 @@
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C36" s="33">
+        <v>33</v>
+      </c>
+      <c r="C36" s="30">
         <v>5</v>
       </c>
-      <c r="D36" s="31">
+      <c r="D36" s="28">
         <v>15000</v>
       </c>
-      <c r="E36" s="22" t="s">
+      <c r="E36" s="20" t="s">
         <v>32</v>
       </c>
       <c r="F36" s="6">
@@ -1174,48 +1196,48 @@
     </row>
     <row r="37" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B37" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" s="33"/>
-      <c r="D37" s="31">
-        <f>54000+5000</f>
-        <v>59000</v>
-      </c>
-      <c r="E37" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C37" s="30"/>
+      <c r="D37" s="28">
+        <f>65880+5000</f>
+        <v>70880</v>
+      </c>
+      <c r="E37" s="20" t="s">
         <v>32</v>
       </c>
       <c r="F37" s="6">
         <f>D37</f>
-        <v>59000</v>
+        <v>70880</v>
       </c>
       <c r="G37" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I37" s="10"/>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="C38" s="22"/>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
       <c r="F38" s="6">
         <f>F39</f>
         <v>220000</v>
       </c>
     </row>
     <row r="39" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="34" t="s">
+      <c r="B39" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="32">
+      <c r="C39" s="29">
         <v>3</v>
       </c>
       <c r="D39" s="7">
         <v>220000</v>
       </c>
-      <c r="E39" s="22"/>
+      <c r="E39" s="20"/>
       <c r="F39" s="6">
         <f>D39</f>
         <v>220000</v>
@@ -1225,12 +1247,12 @@
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
       <c r="F40" s="6">
         <f>C8*C6</f>
         <v>60000</v>
@@ -1241,6 +1263,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="47" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync Oktoberfest budget for 2026-10-23
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D343EF1A-77EF-4541-A592-633788F8BD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF401E47-3D68-4B36-8933-7C6EFAC1F412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -845,7 +845,7 @@
       <c r="E11" s="13"/>
       <c r="F11" s="32">
         <f>F14-F19</f>
-        <v>7281911.0638297871</v>
+        <v>7256379.1489361702</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -914,7 +914,7 @@
       <c r="E18" s="23"/>
       <c r="F18" s="34">
         <f>F19</f>
-        <v>5218088.9361702129</v>
+        <v>5243620.8510638298</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.35">
@@ -926,7 +926,7 @@
       <c r="E19" s="24"/>
       <c r="F19" s="25">
         <f>F20+F21+F22+F23+F24+F38+F40+F29+F34+F35+F36+F37</f>
-        <v>5218088.9361702129</v>
+        <v>5243620.8510638298</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.35">
@@ -1071,7 +1071,7 @@
       <c r="E29" s="28"/>
       <c r="F29" s="6">
         <f>SUM(F30:F33)</f>
-        <v>219148.93617021281</v>
+        <v>244680.85106382982</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.35">
@@ -1133,7 +1133,7 @@
         <v>24</v>
       </c>
       <c r="C33" s="30">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D33" s="28">
         <v>2000</v>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F33" s="7">
         <f>((C33*D33)*6)/0.94</f>
-        <v>25531.914893617024</v>
+        <v>51063.829787234048</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Refresh Oktoberfest budget workbook
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF401E47-3D68-4B36-8933-7C6EFAC1F412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974C140D-D51A-44D9-85CB-79CA8290D89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Средний чек</t>
   </si>
@@ -107,9 +107,6 @@
     <t>Ведущий (13 часов)</t>
   </si>
   <si>
-    <t>Аниматоры (по 5 часов)</t>
-  </si>
-  <si>
     <t>Мастер классы (аниматоры 6 часов)</t>
   </si>
   <si>
@@ -150,6 +147,12 @@
   </si>
   <si>
     <t>Покупка/аренда декора в зону сцены ( бочки-столы (8шт), гирлянда)</t>
+  </si>
+  <si>
+    <t>за 2 дня</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Аниматоры интерактивов </t>
   </si>
 </sst>
 </file>
@@ -799,7 +802,7 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="3">
         <v>0.46</v>
@@ -953,7 +956,7 @@
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C22" s="27"/>
       <c r="D22" s="28">
@@ -1001,7 +1004,7 @@
         <v>6500</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F25" s="7">
         <f>(D25*C25)*1.46*C6</f>
@@ -1019,7 +1022,7 @@
         <v>4000</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F26" s="7">
         <f>(D26*C26)*1.46*C6</f>
@@ -1037,7 +1040,7 @@
         <v>4000</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F27" s="7">
         <f>(D27*C27)*1.46*C6</f>
@@ -1055,7 +1058,7 @@
         <v>4500</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F28" s="7">
         <f>(D28*C28)*1.46*C6</f>
@@ -1094,7 +1097,7 @@
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B31" s="20" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C31" s="30">
         <v>4</v>
@@ -1112,7 +1115,7 @@
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C32" s="30">
         <v>1</v>
@@ -1130,7 +1133,7 @@
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B33" s="20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C33" s="30">
         <v>4</v>
@@ -1148,18 +1151,23 @@
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B34" s="20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C34" s="20"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="20"/>
+      <c r="D34" s="28">
+        <v>50000</v>
+      </c>
+      <c r="E34" s="20" t="s">
+        <v>37</v>
+      </c>
       <c r="F34" s="6">
+        <f>D34</f>
         <v>50000</v>
       </c>
     </row>
     <row r="35" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B35" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="28">
@@ -1167,7 +1175,7 @@
         <v>187000</v>
       </c>
       <c r="E35" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F35" s="6">
         <f>D35</f>
@@ -1177,7 +1185,7 @@
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" s="30">
         <v>5</v>
@@ -1186,7 +1194,7 @@
         <v>15000</v>
       </c>
       <c r="E36" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F36" s="6">
         <f>D36</f>
@@ -1196,7 +1204,7 @@
     </row>
     <row r="37" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B37" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C37" s="30"/>
       <c r="D37" s="28">
@@ -1204,20 +1212,20 @@
         <v>70880</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F37" s="6">
         <f>D37</f>
         <v>70880</v>
       </c>
       <c r="G37" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I37" s="10"/>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B38" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C38" s="20"/>
       <c r="D38" s="20"/>
@@ -1229,7 +1237,7 @@
     </row>
     <row r="39" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="31" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C39" s="29">
         <v>3</v>
@@ -1243,7 +1251,7 @@
         <v>220000</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Refresh October festival budget
</commit_message>
<xml_diff>
--- a/dist/Бюджет Октоберфест.xlsx
+++ b/dist/Бюджет Октоберфест.xlsx
@@ -2,24 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Октоберфест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974C140D-D51A-44D9-85CB-79CA8290D89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5CFFD1-B88F-4A92-BDBB-0F625AE94D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C4098E21-8114-453D-B14B-0A5D84D90A8A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Октоберфест" sheetId="1" r:id="rId1"/>
+    <sheet name="Факт" sheetId="2" r:id="rId2"/>
+    <sheet name="Свод" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -35,8 +34,32 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="D31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Источник: сообщение Кристины от 2026-10-26. За всех аниматоров оплачено 158 537,00 ₽, включая НДС 6%. Расчётное распределение по заложенным человеко-часам: интерактивы 4 × 5 × 3 = 60, мастер-классы 4 × 6 = 24. Общая ставка включает НДС; повторное увеличение на налог не применяется. Фактическая разбивка оплаты по группам не предоставлена.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="47">
   <si>
     <t>Средний чек</t>
   </si>
@@ -47,9 +70,15 @@
     <t>СС фуд</t>
   </si>
   <si>
+    <t>налоги на ФОТ ФУД (*1,46)</t>
+  </si>
+  <si>
     <t>Дней работы</t>
   </si>
   <si>
+    <t>Аниматоры</t>
+  </si>
+  <si>
     <t>Призовой фонд в день</t>
   </si>
   <si>
@@ -74,12 +103,21 @@
     <t>Реклама и продвижение (VK)</t>
   </si>
   <si>
+    <t>Изготовление и поставка рекламного баннера</t>
+  </si>
+  <si>
+    <t>Изготовление билетов и купонов (с доставкой)</t>
+  </si>
+  <si>
     <t>ФОТ ФУД</t>
   </si>
   <si>
     <t>Повара</t>
   </si>
   <si>
+    <t>смена</t>
+  </si>
+  <si>
     <t>Клининг</t>
   </si>
   <si>
@@ -92,83 +130,93 @@
     <t>Ивенты ФОТ</t>
   </si>
   <si>
+    <t>Ведущий (13 часов)</t>
+  </si>
+  <si>
     <t>час</t>
   </si>
   <si>
+    <t xml:space="preserve">Аниматоры интерактивов </t>
+  </si>
+  <si>
+    <t>минус</t>
+  </si>
+  <si>
+    <t>Диджей (2 часа)</t>
+  </si>
+  <si>
+    <t>Мастер классы (аниматоры 6 часов)</t>
+  </si>
+  <si>
+    <t>Мастер классы (расходники на 2 дня)</t>
+  </si>
+  <si>
+    <t>за 2 дня</t>
+  </si>
+  <si>
+    <t>Аренда оборудования (для ведущего и диджея) за три дня</t>
+  </si>
+  <si>
+    <t>за 3 дня</t>
+  </si>
+  <si>
+    <t>Покупка костюмов аниматорам+ведущий</t>
+  </si>
+  <si>
+    <t>Покупка/аренда декора в зону сцены ( бочки-столы (8шт), гирлянда)</t>
+  </si>
+  <si>
+    <t>сено берем у альпак</t>
+  </si>
+  <si>
+    <t>Оборудование ФУД</t>
+  </si>
+  <si>
+    <t>Стоимость гриля (за 3 шт)</t>
+  </si>
+  <si>
+    <t>Покупаем один раз и используем на всех фестивалях</t>
+  </si>
+  <si>
     <t>Призовой фонд</t>
   </si>
   <si>
-    <t>Изготовление и поставка рекламного баннера</t>
-  </si>
-  <si>
-    <t>Аниматоры</t>
-  </si>
-  <si>
-    <t>Ведущий (13 часов)</t>
-  </si>
-  <si>
-    <t>Мастер классы (аниматоры 6 часов)</t>
-  </si>
-  <si>
-    <t>Мастер классы (расходники на 2 дня)</t>
-  </si>
-  <si>
-    <t>Оборудование ФУД</t>
-  </si>
-  <si>
-    <t>Стоимость гриля (за 3 шт)</t>
-  </si>
-  <si>
-    <t>налоги на ФОТ ФУД (*1,46)</t>
-  </si>
-  <si>
-    <t>смена</t>
-  </si>
-  <si>
-    <t>Покупаем один раз и используем на всех фестивалях</t>
-  </si>
-  <si>
-    <t>Аренда оборудования (для ведущего и диджея) за три дня</t>
-  </si>
-  <si>
-    <t>за 3 дня</t>
-  </si>
-  <si>
-    <t>Покупка костюмов аниматорам+ведущий</t>
-  </si>
-  <si>
-    <t>сено берем у альпак</t>
-  </si>
-  <si>
-    <t>Изготовление билетов и купонов (с доставкой)</t>
-  </si>
-  <si>
-    <t>Диджей (2 часа)</t>
-  </si>
-  <si>
-    <t>Покупка/аренда декора в зону сцены ( бочки-столы (8шт), гирлянда)</t>
-  </si>
-  <si>
-    <t>за 2 дня</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аниматоры интерактивов </t>
+    <t>вед</t>
+  </si>
+  <si>
+    <t>с диджей</t>
+  </si>
+  <si>
+    <t>Реклама и продвижение (яндекс директ и VK)</t>
+  </si>
+  <si>
+    <t>Диджей (3 часа)</t>
+  </si>
+  <si>
+    <t>План</t>
+  </si>
+  <si>
+    <t>Факт</t>
+  </si>
+  <si>
+    <t>Отклонение, ₽
+Факт − План</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;₽&quot;_-;\-* #,##0.00\ &quot;₽&quot;_-;_-* &quot;-&quot;??\ &quot;₽&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00;[Red]\-#,##0.00;0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -176,7 +224,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -184,7 +231,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -193,7 +239,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -201,14 +246,12 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -216,11 +259,18 @@
       <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -229,26 +279,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="9" tint="0.59993285927915285"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="5" tint="0.79992065187536243"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="8" tint="0.79992065187536243"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -389,7 +443,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -443,11 +497,54 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="6" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Денежный" xfId="1" builtinId="4"/>
+    <cellStyle name="Денежный" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Процентный" xfId="2" builtinId="5"/>
+    <cellStyle name="Процентный" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -460,6 +557,168 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>501650</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1026" name="Text Box 2" hidden="1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F4FBB7C-38AB-8404-D143-1FD8136B6D35}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1">
+          <a:spLocks noSelect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6350000" cy="6350000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>501650</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71FE86BE-6B7B-F266-6624-48057B4D645E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6350000" cy="6350000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>501650</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{537FAA02-38CF-2DAB-4D1E-2C14D3394037}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6350000" cy="6350000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -505,7 +764,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -557,7 +816,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -618,23 +877,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -644,23 +903,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -668,26 +927,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -722,17 +978,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -749,20 +1005,12 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B06DD981-710B-49F4-BD8B-F9607C12061A}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B2:I42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:I51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="42.54296875" customWidth="1"/>
@@ -771,7 +1019,7 @@
     <col min="5" max="5" width="12.26953125" customWidth="1"/>
     <col min="6" max="6" width="18.54296875" customWidth="1"/>
     <col min="7" max="7" width="69.7265625" customWidth="1"/>
-    <col min="9" max="9" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
@@ -802,7 +1050,7 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="C5" s="3">
         <v>0.46</v>
@@ -812,7 +1060,7 @@
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6">
         <v>3</v>
@@ -820,7 +1068,7 @@
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -828,7 +1076,7 @@
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2">
         <v>20000</v>
@@ -836,12 +1084,12 @@
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
     </row>
-    <row r="10" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="F10" s="4"/>
     </row>
-    <row r="11" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B11" s="12" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
@@ -851,16 +1099,16 @@
         <v>7256379.1489361702</v>
       </c>
     </row>
-    <row r="12" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
       <c r="F12" s="15"/>
     </row>
-    <row r="13" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B13" s="16" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
@@ -872,7 +1120,7 @@
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C14" s="18"/>
       <c r="D14" s="18"/>
@@ -884,7 +1132,7 @@
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="20" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
@@ -901,16 +1149,16 @@
       <c r="E16" s="21"/>
       <c r="F16" s="20"/>
     </row>
-    <row r="17" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B17" s="21"/>
       <c r="C17" s="21"/>
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
       <c r="F17" s="21"/>
     </row>
-    <row r="18" spans="2:6" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B18" s="22" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="23"/>
@@ -920,9 +1168,9 @@
         <v>5243620.8510638298</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B19" s="24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C19" s="24"/>
       <c r="D19" s="24"/>
@@ -932,9 +1180,9 @@
         <v>5243620.8510638298</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B20" s="26" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C20" s="27"/>
       <c r="D20" s="27"/>
@@ -943,9 +1191,9 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B21" s="26" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C21" s="27"/>
       <c r="D21" s="27"/>
@@ -954,9 +1202,9 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B22" s="26" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C22" s="27"/>
       <c r="D22" s="28">
@@ -969,9 +1217,9 @@
         <v>9200</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B23" s="20" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
@@ -981,9 +1229,9 @@
         <v>2875000</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B24" s="20" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
@@ -993,9 +1241,9 @@
         <v>1081860</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B25" s="20" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C25" s="29">
         <v>12</v>
@@ -1004,16 +1252,16 @@
         <v>6500</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F25" s="7">
         <f>(D25*C25)*1.46*C6</f>
         <v>341640</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B26" s="20" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C26" s="29">
         <v>6</v>
@@ -1022,16 +1270,16 @@
         <v>4000</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F26" s="7">
         <f>(D26*C26)*1.46*C6</f>
         <v>105120</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B27" s="20" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C27" s="29">
         <v>25</v>
@@ -1040,16 +1288,16 @@
         <v>4000</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F27" s="7">
         <f>(D27*C27)*1.46*C6</f>
         <v>438000</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B28" s="20" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C28" s="29">
         <v>10</v>
@@ -1058,16 +1306,16 @@
         <v>4500</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F28" s="7">
         <f>(D28*C28)*1.46*C6</f>
         <v>197100</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B29" s="20" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C29" s="29"/>
       <c r="D29" s="28"/>
@@ -1077,9 +1325,9 @@
         <v>244680.85106382982</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B30" s="20" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C30" s="29">
         <v>1</v>
@@ -1088,16 +1336,19 @@
         <v>4000</v>
       </c>
       <c r="E30" s="20" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F30" s="7">
         <f>(D30*C30*13)/0.94</f>
         <v>55319.148936170219</v>
       </c>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="I30" s="41">
+        <v>55315</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B31" s="20" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C31" s="30">
         <v>4</v>
@@ -1106,16 +1357,22 @@
         <v>2000</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F31" s="7">
         <f>(D31*C31*5*C6)/0.94</f>
         <v>127659.57446808512</v>
       </c>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="G31" s="40" t="s">
+        <v>26</v>
+      </c>
+      <c r="H31">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B32" s="20" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C32" s="30">
         <v>1</v>
@@ -1124,16 +1381,22 @@
         <v>5000</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" s="7">
+        <v>24</v>
+      </c>
+      <c r="F32" s="65">
         <f>((D32*C32)*2)/0.94</f>
         <v>10638.297872340427</v>
       </c>
+      <c r="H32">
+        <v>5000</v>
+      </c>
+      <c r="I32" s="41">
+        <v>15957</v>
+      </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B33" s="20" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C33" s="30">
         <v>4</v>
@@ -1142,7 +1405,7 @@
         <v>2000</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F33" s="7">
         <f>((C33*D33)*6)/0.94</f>
@@ -1151,23 +1414,27 @@
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B34" s="20" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C34" s="20"/>
       <c r="D34" s="28">
         <v>50000</v>
       </c>
       <c r="E34" s="20" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F34" s="6">
         <f>D34</f>
         <v>50000</v>
       </c>
+      <c r="I34" s="42">
+        <f>40000-I36</f>
+        <v>26064</v>
+      </c>
     </row>
     <row r="35" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B35" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="28">
@@ -1175,17 +1442,23 @@
         <v>187000</v>
       </c>
       <c r="E35" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F35" s="6">
         <f>D35</f>
         <v>187000</v>
       </c>
-      <c r="I35" s="10"/>
+      <c r="H35">
+        <v>10000</v>
+      </c>
+      <c r="I35" s="10">
+        <f>F35+10000</f>
+        <v>197000</v>
+      </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B36" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C36" s="30">
         <v>5</v>
@@ -1194,17 +1467,20 @@
         <v>15000</v>
       </c>
       <c r="E36" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F36" s="6">
         <f>D36</f>
         <v>15000</v>
       </c>
-      <c r="I36" s="10"/>
+      <c r="I36" s="42">
+        <f>8170.71+2593.86+3171.43</f>
+        <v>13936</v>
+      </c>
     </row>
     <row r="37" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B37" s="11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C37" s="30"/>
       <c r="D37" s="28">
@@ -1212,20 +1488,23 @@
         <v>70880</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F37" s="6">
         <f>D37</f>
         <v>70880</v>
       </c>
       <c r="G37" t="s">
-        <v>33</v>
-      </c>
-      <c r="I37" s="10"/>
+        <v>35</v>
+      </c>
+      <c r="I37" s="42">
+        <f>64800+2000</f>
+        <v>66800</v>
+      </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B38" s="20" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="C38" s="20"/>
       <c r="D38" s="20"/>
@@ -1235,9 +1514,9 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="39" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="31" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C39" s="29">
         <v>3</v>
@@ -1251,12 +1530,12 @@
         <v>220000</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B40" s="20" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C40" s="20"/>
       <c r="D40" s="20"/>
@@ -1269,8 +1548,1327 @@
     <row r="42" spans="2:9" x14ac:dyDescent="0.35">
       <c r="F42" s="1"/>
     </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C50" t="s">
+        <v>40</v>
+      </c>
+      <c r="D50">
+        <v>81100</v>
+      </c>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C51" t="s">
+        <v>41</v>
+      </c>
+      <c r="D51">
+        <v>280000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="47" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="B2:F51"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="42.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.7265625" customWidth="1"/>
+    <col min="4" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="12.26953125" customWidth="1"/>
+    <col min="6" max="6" width="18.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="39">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.23</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.46</v>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2">
+        <v>20000</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B11" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="32">
+        <f>F14-F19</f>
+        <v>7362794.3031914895</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="15"/>
+    </row>
+    <row r="13" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B13" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="33">
+        <f>F14</f>
+        <v>12500000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B14" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="19">
+        <f>SUM(F15:F17)</f>
+        <v>12500000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B15" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="7">
+        <f>C2*C3</f>
+        <v>12500000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="20"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+    </row>
+    <row r="18" spans="2:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B18" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="34">
+        <f>F19</f>
+        <v>5137205.6968085105</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="25">
+        <f>F20+F21+F22+F23+F24+F38+F40+F29+F34+F35+F36+F37</f>
+        <v>5137205.6968085105</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B20" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="45">
+        <f>168624.84+158911.41</f>
+        <v>327536.25</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="5">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="27"/>
+      <c r="D22" s="28">
+        <f>6200+500+2500</f>
+        <v>9200</v>
+      </c>
+      <c r="E22" s="27"/>
+      <c r="F22" s="5">
+        <f>D22</f>
+        <v>9200</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="6">
+        <f>C2*C3*C4</f>
+        <v>2875000</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="6">
+        <f>SUM(F25:F28)</f>
+        <v>1081860</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B25" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="29">
+        <v>12</v>
+      </c>
+      <c r="D25" s="28">
+        <v>6500</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" s="7">
+        <f>(D25*C25)*1.46*C6</f>
+        <v>341640</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B26" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="29">
+        <v>6</v>
+      </c>
+      <c r="D26" s="28">
+        <v>4000</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="7">
+        <f>(D26*C26)*1.46*C6</f>
+        <v>105120</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B27" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="29">
+        <v>25</v>
+      </c>
+      <c r="D27" s="28">
+        <v>4000</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="7">
+        <f>(D27*C27)*1.46*C6</f>
+        <v>438000</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B28" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="29">
+        <v>10</v>
+      </c>
+      <c r="D28" s="28">
+        <v>4500</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="7">
+        <f>(D28*C28)*1.46*C6</f>
+        <v>197100</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B29" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="29"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="6">
+        <f>SUM(F30:F33)</f>
+        <v>229809.44680851066</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B30" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="29">
+        <v>1</v>
+      </c>
+      <c r="D30" s="28">
+        <v>4000</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30" s="43">
+        <v>55315</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B31" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="30">
+        <v>4</v>
+      </c>
+      <c r="D31" s="28">
+        <f>158537/(C31*5*$C$6+C33*6)</f>
+        <v>1887.3452380952381</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" s="7">
+        <f>ROUND(D31*C31*5*$C$6,2)</f>
+        <v>113240.71</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B32" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" s="30">
+        <v>1</v>
+      </c>
+      <c r="D32" s="28">
+        <v>5000</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F32" s="64">
+        <f>((D32*C32)*3)/0.94</f>
+        <v>15957.44680851064</v>
+      </c>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B33" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="30">
+        <v>4</v>
+      </c>
+      <c r="D33" s="28">
+        <f>D31</f>
+        <v>1887.3452380952381</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F33" s="7">
+        <f>ROUND(D33*C33*6,2)</f>
+        <v>45296.29</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B34" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="20"/>
+      <c r="D34" s="28">
+        <v>26064</v>
+      </c>
+      <c r="E34" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="F34" s="44">
+        <f>D34</f>
+        <v>26064</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="B35" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C35" s="20"/>
+      <c r="D35" s="28">
+        <f>197000</f>
+        <v>197000</v>
+      </c>
+      <c r="E35" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="F35" s="44">
+        <f>D35</f>
+        <v>197000</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B36" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="30">
+        <v>5</v>
+      </c>
+      <c r="D36" s="28">
+        <f>8170.71+2593.86+3171.43</f>
+        <v>13936</v>
+      </c>
+      <c r="E36" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="44">
+        <f>D36</f>
+        <v>13936</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="29" x14ac:dyDescent="0.35">
+      <c r="B37" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="30"/>
+      <c r="D37" s="28">
+        <f>64800+2000</f>
+        <v>66800</v>
+      </c>
+      <c r="E37" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="F37" s="44">
+        <f>D37</f>
+        <v>66800</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B38" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="6">
+        <f>F39</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="39" spans="2:6" ht="7.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="C39" s="29">
+        <v>3</v>
+      </c>
+      <c r="D39" s="7">
+        <v>220000</v>
+      </c>
+      <c r="E39" s="20"/>
+      <c r="F39" s="6">
+        <f>D39</f>
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B40" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="20"/>
+      <c r="F40" s="6">
+        <f>C8*C6</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="F42" s="1"/>
+    </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C50" t="s">
+        <v>40</v>
+      </c>
+      <c r="D50">
+        <v>81100</v>
+      </c>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C51" t="s">
+        <v>41</v>
+      </c>
+      <c r="D51">
+        <v>280000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A2:G51"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="42.54296875" customWidth="1"/>
+    <col min="2" max="2" width="15.7265625" customWidth="1"/>
+    <col min="3" max="3" width="16.7265625" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" customWidth="1"/>
+    <col min="5" max="5" width="18.54296875" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>2500</v>
+      </c>
+      <c r="F2" s="62">
+        <f>Факт!C2</f>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>5000</v>
+      </c>
+      <c r="F3" s="63">
+        <f>Факт!C3</f>
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0.23</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="F4" s="61">
+        <f>Факт!C4</f>
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.46</v>
+      </c>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="F5" s="61">
+        <f>Факт!C5</f>
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="F6" s="63">
+        <f>Факт!C6</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="F7" s="63">
+        <f>Факт!C7</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2">
+        <v>20000</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="F8" s="63">
+        <f>Факт!C8</f>
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="46" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="32">
+        <f>E14-E19</f>
+        <v>7256379.1489361702</v>
+      </c>
+      <c r="F11" s="47">
+        <f>Факт!F11</f>
+        <v>7362794.3031914895</v>
+      </c>
+      <c r="G11" s="47">
+        <f>F11-E11</f>
+        <v>106415.15425531939</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+    </row>
+    <row r="13" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="33">
+        <f>E14</f>
+        <v>12500000</v>
+      </c>
+      <c r="F13" s="49">
+        <f>Факт!F13</f>
+        <v>12500000</v>
+      </c>
+      <c r="G13" s="49">
+        <f>F13-E13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="19">
+        <f>SUM(E15:E17)</f>
+        <v>12500000</v>
+      </c>
+      <c r="F14" s="50">
+        <f>Факт!F14</f>
+        <v>12500000</v>
+      </c>
+      <c r="G14" s="50">
+        <f>F14-E14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="7">
+        <f>B2*B3</f>
+        <v>12500000</v>
+      </c>
+      <c r="F15" s="51">
+        <f>Факт!F15</f>
+        <v>12500000</v>
+      </c>
+      <c r="G15" s="51">
+        <f>F15-E15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="51"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="52"/>
+      <c r="G17" s="52"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="34">
+        <f>E19</f>
+        <v>5243620.8510638298</v>
+      </c>
+      <c r="F18" s="53">
+        <f>Факт!F18</f>
+        <v>5137205.6968085105</v>
+      </c>
+      <c r="G18" s="53">
+        <f t="shared" ref="G18:G40" si="0">F18-E18</f>
+        <v>-106415.15425531939</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="25">
+        <f>E20+E21+E22+E23+E24+E38+E40+E29+E34+E35+E36+E37</f>
+        <v>5243620.8510638298</v>
+      </c>
+      <c r="F19" s="54">
+        <f>Факт!F19</f>
+        <v>5137205.6968085105</v>
+      </c>
+      <c r="G19" s="54">
+        <f t="shared" si="0"/>
+        <v>-106415.15425531939</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="5">
+        <v>400000</v>
+      </c>
+      <c r="F20" s="55">
+        <f>Факт!F20</f>
+        <v>327536.25</v>
+      </c>
+      <c r="G20" s="55">
+        <f t="shared" si="0"/>
+        <v>-72463.75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="5">
+        <v>30000</v>
+      </c>
+      <c r="F21" s="56">
+        <f>Факт!F21</f>
+        <v>30000</v>
+      </c>
+      <c r="G21" s="56">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="27"/>
+      <c r="C22" s="28">
+        <f>6200+500+2500</f>
+        <v>9200</v>
+      </c>
+      <c r="D22" s="27"/>
+      <c r="E22" s="5">
+        <f>C22</f>
+        <v>9200</v>
+      </c>
+      <c r="F22" s="56">
+        <f>Факт!F22</f>
+        <v>9200</v>
+      </c>
+      <c r="G22" s="56">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="6">
+        <f>B2*B3*B4</f>
+        <v>2875000</v>
+      </c>
+      <c r="F23" s="57">
+        <f>Факт!F23</f>
+        <v>2875000</v>
+      </c>
+      <c r="G23" s="57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="6">
+        <f>SUM(E25:E28)</f>
+        <v>1081860</v>
+      </c>
+      <c r="F24" s="57">
+        <f>Факт!F24</f>
+        <v>1081860</v>
+      </c>
+      <c r="G24" s="57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="29">
+        <v>12</v>
+      </c>
+      <c r="C25" s="28">
+        <v>6500</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="7">
+        <f>(C25*B25)*1.46*B6</f>
+        <v>341640</v>
+      </c>
+      <c r="F25" s="51">
+        <f>Факт!F25</f>
+        <v>341640</v>
+      </c>
+      <c r="G25" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="29">
+        <v>6</v>
+      </c>
+      <c r="C26" s="28">
+        <v>4000</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="7">
+        <f>(C26*B26)*1.46*B6</f>
+        <v>105120</v>
+      </c>
+      <c r="F26" s="51">
+        <f>Факт!F26</f>
+        <v>105120</v>
+      </c>
+      <c r="G26" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="29">
+        <v>25</v>
+      </c>
+      <c r="C27" s="28">
+        <v>4000</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" s="7">
+        <f>(C27*B27)*1.46*B6</f>
+        <v>438000</v>
+      </c>
+      <c r="F27" s="51">
+        <f>Факт!F27</f>
+        <v>438000</v>
+      </c>
+      <c r="G27" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="29">
+        <v>10</v>
+      </c>
+      <c r="C28" s="28">
+        <v>4500</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E28" s="7">
+        <f>(C28*B28)*1.46*B6</f>
+        <v>197100</v>
+      </c>
+      <c r="F28" s="51">
+        <f>Факт!F28</f>
+        <v>197100</v>
+      </c>
+      <c r="G28" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" s="29"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="6">
+        <f>SUM(E30:E33)</f>
+        <v>244680.85106382982</v>
+      </c>
+      <c r="F29" s="57">
+        <f>Факт!F29</f>
+        <v>229809.44680851066</v>
+      </c>
+      <c r="G29" s="57">
+        <f t="shared" si="0"/>
+        <v>-14871.404255319154</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="29">
+        <v>1</v>
+      </c>
+      <c r="C30" s="28">
+        <v>4000</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" s="7">
+        <f>(C30*B30*13)/0.94</f>
+        <v>55319.148936170219</v>
+      </c>
+      <c r="F30" s="58">
+        <f>Факт!F30</f>
+        <v>55315</v>
+      </c>
+      <c r="G30" s="58">
+        <f t="shared" si="0"/>
+        <v>-4.1489361702188035</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="30">
+        <v>4</v>
+      </c>
+      <c r="C31" s="28">
+        <v>2000</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="7">
+        <f>(C31*B31*5*B6)/0.94</f>
+        <v>127659.57446808512</v>
+      </c>
+      <c r="F31" s="51">
+        <f>Факт!F31</f>
+        <v>113240.71</v>
+      </c>
+      <c r="G31" s="51">
+        <f t="shared" si="0"/>
+        <v>-14418.864468085114</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="39" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B32" s="36">
+        <v>1</v>
+      </c>
+      <c r="C32" s="37">
+        <v>5000</v>
+      </c>
+      <c r="D32" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="E32" s="38">
+        <f>((C32*B32)*2)/0.94</f>
+        <v>10638.297872340427</v>
+      </c>
+      <c r="F32" s="59">
+        <f>Факт!F32</f>
+        <v>15957.44680851064</v>
+      </c>
+      <c r="G32" s="59">
+        <f t="shared" si="0"/>
+        <v>5319.1489361702133</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="30">
+        <v>4</v>
+      </c>
+      <c r="C33" s="28">
+        <v>2000</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E33" s="7">
+        <f>((B33*C33)*6)/0.94</f>
+        <v>51063.829787234048</v>
+      </c>
+      <c r="F33" s="51">
+        <f>Факт!F33</f>
+        <v>45296.29</v>
+      </c>
+      <c r="G33" s="51">
+        <f t="shared" si="0"/>
+        <v>-5767.5397872340473</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" s="20"/>
+      <c r="C34" s="28">
+        <v>50000</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E34" s="6">
+        <f>C34</f>
+        <v>50000</v>
+      </c>
+      <c r="F34" s="60">
+        <f>Факт!F34</f>
+        <v>26064</v>
+      </c>
+      <c r="G34" s="60">
+        <f t="shared" si="0"/>
+        <v>-23936</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="20"/>
+      <c r="C35" s="28">
+        <f>187000</f>
+        <v>187000</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E35" s="6">
+        <f>C35</f>
+        <v>187000</v>
+      </c>
+      <c r="F35" s="60">
+        <f>Факт!F35</f>
+        <v>197000</v>
+      </c>
+      <c r="G35" s="60">
+        <f t="shared" si="0"/>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="30">
+        <v>5</v>
+      </c>
+      <c r="C36" s="28">
+        <v>15000</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E36" s="6">
+        <f>C36</f>
+        <v>15000</v>
+      </c>
+      <c r="F36" s="60">
+        <f>Факт!F36</f>
+        <v>13936</v>
+      </c>
+      <c r="G36" s="60">
+        <f t="shared" si="0"/>
+        <v>-1064</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="30"/>
+      <c r="C37" s="28">
+        <f>65880+5000</f>
+        <v>70880</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="E37" s="6">
+        <f>C37</f>
+        <v>70880</v>
+      </c>
+      <c r="F37" s="60">
+        <f>Факт!F37</f>
+        <v>66800</v>
+      </c>
+      <c r="G37" s="60">
+        <f t="shared" si="0"/>
+        <v>-4080</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="20"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="20"/>
+      <c r="E38" s="6">
+        <f>E39</f>
+        <v>220000</v>
+      </c>
+      <c r="F38" s="57">
+        <f>Факт!F38</f>
+        <v>220000</v>
+      </c>
+      <c r="G38" s="57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="7.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" s="29">
+        <v>3</v>
+      </c>
+      <c r="C39" s="7">
+        <v>220000</v>
+      </c>
+      <c r="D39" s="20"/>
+      <c r="E39" s="6">
+        <f>C39</f>
+        <v>220000</v>
+      </c>
+      <c r="F39" s="57">
+        <f>Факт!F39</f>
+        <v>220000</v>
+      </c>
+      <c r="G39" s="57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="6">
+        <f>B8*B6</f>
+        <v>60000</v>
+      </c>
+      <c r="F40" s="57">
+        <f>Факт!F40</f>
+        <v>60000</v>
+      </c>
+      <c r="G40" s="57">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B50" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50">
+        <v>81100</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B51" t="s">
+        <v>41</v>
+      </c>
+      <c r="C51">
+        <v>280000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>